<commit_message>
Add Stage 8: regression tests for lending bug-fix stages
</commit_message>
<xml_diff>
--- a/tests/fixtures/excel/09_old_display_name.xlsx
+++ b/tests/fixtures/excel/09_old_display_name.xlsx
@@ -466,7 +466,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>05-Feb-24 | ₹50,000 | Due 10</t>
+          <t>01-Mar-24 | ₹50,000 | Due 10</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>05-Feb-24 | ₹40,000 | Due 10</t>
+          <t>01-Mar-24 | ₹40,000 | Due 10</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -519,7 +519,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>display name after principal repayment (mutated)</t>
+          <t>display name using outstanding (must not silently match)</t>
         </is>
       </c>
     </row>

</xml_diff>